<commit_message>
changed design rules acc. to 2 oz restrictions of jlc. all 0.3 mm traces down to 0.2 mm and corrected placement and routing for having 0.2 mm spacing everywhere. Regenerated Output Files. THIS IS THE PRODUCED REVISION AT JLCPCB
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_SiC_inverter_828xcc/Rev01/BOM/BOM_JLC-UZ_PER_SiC_inverter_828xcc.xlsx
+++ b/Project Outputs for UZ_PER_SiC_inverter_828xcc/Rev01/BOM/BOM_JLC-UZ_PER_SiC_inverter_828xcc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_sic_inverter_828xcc\Project Outputs for UZ_PER_SiC_inverter_828xcc\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F361966-186C-4F4F-B994-447BBDA05E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5768D4D8-ABFF-4CC8-BE63-A7F25A6EF4A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="74055" yWindow="15" windowWidth="19125" windowHeight="10035" xr2:uid="{E740077A-DE3A-4E71-8ADE-FB65A92BCC9A}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{2B279F93-689D-4597-BA69-2775D0F7490C}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_SiC_inverter_828" sheetId="1" r:id="rId1"/>
@@ -650,7 +650,7 @@
     <t>R1, R2</t>
   </si>
   <si>
-    <t xml:space="preserve">KOA Speer	</t>
+    <t>KOA Speer</t>
   </si>
   <si>
     <t>SMD resistor E24 series</t>
@@ -1302,7 +1302,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9225DD1A-2D23-4E40-B9C7-97A3E5E7729D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A37BEA-836C-4387-BF0A-90D36726FEC3}">
   <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>